<commit_message>
Update workbook with three sheets and add XML analysis to README
- Protected: formulas stuck as #NAME? on protected sheet
- Unprotected: formulas stuck as #NAME? on unprotected sheet
- Correct: formulas properly resolved with add-in loaded

README now includes underlying XML showing the _xldudf_ rewrite
that occurs when formulas are properly recognized vs stuck.
</commit_message>
<xml_diff>
--- a/Custom Functions Protected Sheet Repro.xlsx
+++ b/Custom Functions Protected Sheet Repro.xlsx
@@ -8,13 +8,14 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/enelson/dev/project-notes/xconnect-core-migration-testing/repro-protected-sheet-custom-functions/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3EC3B501-0D40-A34B-A29A-89C769463C58}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2E635EE8-1492-7849-955F-9DD047D080CB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1100" yWindow="900" windowWidth="28040" windowHeight="17180" activeTab="1" xr2:uid="{DB220A69-93A6-F24B-919C-F8D33D144390}"/>
+    <workbookView xWindow="1100" yWindow="900" windowWidth="28040" windowHeight="17180" activeTab="2" xr2:uid="{DB220A69-93A6-F24B-919C-F8D33D144390}"/>
   </bookViews>
   <sheets>
     <sheet name="Protected" sheetId="1" r:id="rId1"/>
     <sheet name="Unprotected" sheetId="2" r:id="rId2"/>
+    <sheet name="Correct" sheetId="3" r:id="rId3"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -37,7 +38,7 @@
 </file>
 
 <file path=xl/metadata.xml><?xml version="1.0" encoding="utf-8"?>
-<metadata xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xda="http://schemas.microsoft.com/office/spreadsheetml/2017/dynamicarray">
+<metadata xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xlrd="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata" xmlns:xda="http://schemas.microsoft.com/office/spreadsheetml/2017/dynamicarray">
   <metadataTypes count="1">
     <metadataType name="XLDAPR" minSupportedVersion="120000" copy="1" pasteAll="1" pasteValues="1" merge="1" splitFirst="1" rowColShift="1" clearFormats="1" clearComments="1" assign="1" coerce="1" cellMeta="1"/>
   </metadataTypes>
@@ -423,6 +424,32 @@
 </a:theme>
 </file>
 
+<file path=xl/webextensions/taskpanes.xml><?xml version="1.0" encoding="utf-8"?>
+<wetp:taskpanes xmlns:wetp="http://schemas.microsoft.com/office/webextensions/taskpanes/2010/11">
+  <wetp:taskpane dockstate="right" visibility="0" width="0" row="0">
+    <wetp:webextensionref xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+  </wetp:taskpane>
+</wetp:taskpanes>
+</file>
+
+<file path=xl/webextensions/webextension1.xml><?xml version="1.0" encoding="utf-8"?>
+<we:webextension xmlns:we="http://schemas.microsoft.com/office/webextensions/webextension/2010/11" id="{88C9DF49-DEB8-0D4E-B730-E4053453480D}">
+  <we:reference id="00000000-0000-0000-0000-000000000001" version="1.0.0.0" store="developer" storeType="Registry"/>
+  <we:alternateReferences/>
+  <we:properties/>
+  <we:bindings/>
+  <we:snapshot xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships"/>
+  <we:extLst>
+    <a:ext xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" uri="{7C84B067-C214-45C3-A712-C9D94CD141B2}">
+      <we:customFunctionIdList>
+        <we:customFunctionIds>_xldudf_CONTOSO_ADD</we:customFunctionIds>
+        <we:customFunctionIds>_xldudf_CONTOSO_GET</we:customFunctionIds>
+      </we:customFunctionIdList>
+    </a:ext>
+  </we:extLst>
+</we:webextension>
+</file>
+
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{91D54C53-9028-5346-8002-FD6CA0EBB842}">
   <dimension ref="A1:B1"/>
@@ -462,4 +489,24 @@
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9866641C-DF50-AC4A-9213-3D6DB67A28CE}">
+  <dimension ref="A1:B1"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <sheetData>
+    <row r="1" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A1" cm="1">
+        <f t="array" ref="A1">_xldudf_CONTOSO_ADD(1,2)</f>
+        <v>3</v>
+      </c>
+      <c r="B1" t="str" cm="1">
+        <f t="array" ref="B1">_xldudf_CONTOSO_GET("test")</f>
+        <v>test</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>